<commit_message>
data: daily plan snapshot [2026-04-07]
</commit_message>
<xml_diff>
--- a/data/changelog.xlsx
+++ b/data/changelog.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1181,6 +1181,636 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Paid (30d)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Turbo 10 GB</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Monthly Price (R$)</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Paid (30d)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Turbo 10 GB</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Base Plan GB</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>TIM</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Paid (30d)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>TIM Pré XIP Plus</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Monthly Price (R$)</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>TIM</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Paid (30d)</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>TIM Pré XIP Plus</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Base Plan GB</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Claro</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Paid (30d)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Claro Prezão</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Monthly Price (R$)</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Claro</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Pre-Paid (30d)</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Claro Prezão</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Base Plan GB</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Controle</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Controle 21 GB</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Base Plan GB</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>TIM</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Controle</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>TIM Controle</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Monthly Price (R$)</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>43.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>TIM</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Controle</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>TIM Controle</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Base Plan GB</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Claro</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Controle</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Claro Controle</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Monthly Price (R$)</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>59.9</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Vivo</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Post-Paid</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Vivo Pós — Entry</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Monthly Price (R$)</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>140.0</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>133.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>TIM</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Post-Paid</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>TIM Black A</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Monthly Price (R$)</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>159.99</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>119.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>TIM</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Post-Paid</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>TIM Black A</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Base Plan GB</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Claro</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Post-Paid</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Claro Pós 70 GB</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Monthly Price (R$)</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>119.9</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>119.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Claro</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Post-Paid</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Claro Pós 70 GB</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Base Plan GB</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>